<commit_message>
Confirm R-1 as Ebara screw chiller RHS DW202M2 from nameplate
Nameplate (エバラスクリュー冷凍機, 荏原冷熱システム, 2014/12) confirms the 36/37F
local chiller is a single water-cooled SCREW machine, model RHS DW202M2:
370 kW cooling / 82.2 kW input (COP 4.5), twin 45 kW screw compressors,
dual HFC-407C circuits. Updated device type, R-1.KW basis, docstring, cover,
legend and README to the confirmed type/model; regenerated the workbook.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Red5-DHCP_BMS_IO_List.xlsx
+++ b/Red5-DHCP_BMS_IO_List.xlsx
@@ -628,7 +628,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>R-1 single water-cooled chiller (Ebara ~370 kW, COP 4.51) in changeover with DHC via HEX-1 + CP-8; CDP-3 + CT-3 condenser; CP-7 CHW; HP-4 + EX4 + EXT-3 secondary; 2 source-changeover valves</t>
+          <t>R-1 single water-cooled SCREW chiller (Ebara RHS DW202M2, 370 kW / 82.2 kW in / COP 4.5, twin 45 kW screw comp, R-407C) in changeover with DHC via HEX-1 + CP-8; CDP-3 + CT-3 condenser; CP-7 CHW; HP-4 + EX4 + EXT-3 secondary; 2 source-changeover valves</t>
         </is>
       </c>
     </row>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="D283" s="8" t="inlineStr">
         <is>
-          <t>Water-cooled chiller (local backup)</t>
+          <t>Water-cooled screw chiller (local backup)</t>
         </is>
       </c>
       <c r="E283" s="8" t="inlineStr">
@@ -21816,7 +21816,7 @@
       </c>
       <c r="D284" s="8" t="inlineStr">
         <is>
-          <t>Water-cooled chiller (local backup)</t>
+          <t>Water-cooled screw chiller (local backup)</t>
         </is>
       </c>
       <c r="E284" s="8" t="inlineStr">
@@ -21881,7 +21881,7 @@
       </c>
       <c r="D285" s="8" t="inlineStr">
         <is>
-          <t>Water-cooled chiller (local backup)</t>
+          <t>Water-cooled screw chiller (local backup)</t>
         </is>
       </c>
       <c r="E285" s="8" t="inlineStr">
@@ -21942,7 +21942,7 @@
       </c>
       <c r="D286" s="8" t="inlineStr">
         <is>
-          <t>Water-cooled chiller (local backup)</t>
+          <t>Water-cooled screw chiller (local backup)</t>
         </is>
       </c>
       <c r="E286" s="8" t="inlineStr">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="D287" s="8" t="inlineStr">
         <is>
-          <t>Water-cooled chiller (local backup)</t>
+          <t>Water-cooled screw chiller (local backup)</t>
         </is>
       </c>
       <c r="E287" s="8" t="inlineStr">
@@ -22080,7 +22080,7 @@
       </c>
       <c r="D288" s="8" t="inlineStr">
         <is>
-          <t>Water-cooled chiller (local backup)</t>
+          <t>Water-cooled screw chiller (local backup)</t>
         </is>
       </c>
       <c r="E288" s="8" t="inlineStr">
@@ -22153,7 +22153,7 @@
       </c>
       <c r="D289" s="8" t="inlineStr">
         <is>
-          <t>Water-cooled chiller (local backup)</t>
+          <t>Water-cooled screw chiller (local backup)</t>
         </is>
       </c>
       <c r="E289" s="8" t="inlineStr">
@@ -22222,7 +22222,7 @@
       </c>
       <c r="D290" s="8" t="inlineStr">
         <is>
-          <t>Water-cooled chiller (local backup)</t>
+          <t>Water-cooled screw chiller (local backup)</t>
         </is>
       </c>
       <c r="E290" s="8" t="inlineStr">
@@ -22287,7 +22287,7 @@
       </c>
       <c r="D291" s="8" t="inlineStr">
         <is>
-          <t>Water-cooled chiller (local backup)</t>
+          <t>Water-cooled screw chiller (local backup)</t>
         </is>
       </c>
       <c r="E291" s="8" t="inlineStr">
@@ -22334,7 +22334,7 @@
       </c>
       <c r="O291" s="8" t="inlineStr">
         <is>
-          <t>For COP; nameplate 370 kW / COP 4.51</t>
+          <t>Ebara screw RHS DW202M2: 370 kW cool / 82.2 kW in (COP 4.5); 2×45 kW screw comp, R-407C</t>
         </is>
       </c>
     </row>
@@ -22356,7 +22356,7 @@
       </c>
       <c r="D292" s="8" t="inlineStr">
         <is>
-          <t>Water-cooled chiller (local backup)</t>
+          <t>Water-cooled screw chiller (local backup)</t>
         </is>
       </c>
       <c r="E292" s="8" t="inlineStr">
@@ -80985,7 +80985,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Local 36/37F water-cooled chiller (Ebara ~370 kW, COP 4.51), DHC-backup</t>
+          <t>Local 36/37F water-cooled SCREW chiller — Ebara RHS DW202M2 (370 kW, COP 4.5, twin screw, R-407C), DHC-backup</t>
         </is>
       </c>
     </row>

</xml_diff>